<commit_message>
Add base path for GitHub Pages deployment
</commit_message>
<xml_diff>
--- a/hydrant-flow-test-calculator.xlsx
+++ b/hydrant-flow-test-calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6f711bccef12e9ca/Desktop/hydrant-flow-test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="179" documentId="8_{599F4E0A-716C-4BD1-9B12-647D936C6E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C564E2B3-034F-4DDE-8287-B2F974556572}"/>
+  <xr:revisionPtr revIDLastSave="181" documentId="8_{599F4E0A-716C-4BD1-9B12-647D936C6E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B69FBCA-3FA2-4A0C-9EB6-C84C6B97A439}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="165" windowWidth="29040" windowHeight="15720" xr2:uid="{C44C67A6-7468-4286-A2CC-CA4FEFA488D0}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Estimated Flow" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" calcCompleted="0"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2141,7 +2141,7 @@
   <dimension ref="A1:E83"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.6328125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="30.6328125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.6328125" customWidth="1"/>
     <col min="4" max="5" width="25.6328125" style="1" customWidth="1"/>
   </cols>

</xml_diff>